<commit_message>
文档结构预分析: init 生成 document_summary, next 嵌入 batch JSON
</commit_message>
<xml_diff>
--- a/data/term_base.xlsx
+++ b/data/term_base.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -455,6 +455,40 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>アミーゴ</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>朋友</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>西班牙语 amigo 音译。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>カラ</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>卡拉</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>人名，音译。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>